<commit_message>
Add Responses to the questions
</commit_message>
<xml_diff>
--- a/mia07_t3_tra_resultados_viterbi.xlsx
+++ b/mia07_t3_tra_resultados_viterbi.xlsx
@@ -473,7 +473,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>AQ0MS0</t>
+          <t>NCFS000</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -486,7 +486,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>1.295582484193506e-09</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -535,14 +535,14 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>SPS00</t>
+          <t>Fp</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1.988063133517315e-05</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -554,19 +554,19 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>5.440257583147429e-12</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>3.529518322132861e-16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>NCFS000</t>
+          <t>DA0MS0</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -576,7 +576,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>2.779888150251198e-06</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -597,7 +597,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>NCMS000</t>
+          <t>NCMP000</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -610,7 +610,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>2.827818374535177e-08</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -619,7 +619,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>4.107075865754602e-15</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -628,11 +628,11 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>VMIP3S0</t>
+          <t>NCMS000</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0012941074971961</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -641,7 +641,7 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>2.827818374535177e-08</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -659,17 +659,17 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>DA0MS0</t>
+          <t>VMIP3S0</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>0.0012941074971961</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>2.779888150251198e-06</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -690,7 +690,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>NCMP000</t>
+          <t>AQ0MS0</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -703,7 +703,7 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1.295582484193506e-09</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -712,7 +712,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>4.107075865754602e-15</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -721,14 +721,14 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Fp</t>
+          <t>SPS00</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1.988063133517315e-05</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -740,13 +740,13 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>5.440257583147429e-12</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>3.529518322132861e-16</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>